<commit_message>
Final commit before final cleanup
Final commit before final cleanup
</commit_message>
<xml_diff>
--- a/data/test/Example_Q_and_A_for_RAG_LLM.xlsx
+++ b/data/test/Example_Q_and_A_for_RAG_LLM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\00_SW\01_RAG\data\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5237B2-B70E-4B68-9EEF-C47DA6D649CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233044DC-DB70-4DC4-885A-E7C7A6171E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2AFBA614-42DE-4065-86FD-C0FD95C7E89C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{2AFBA614-42DE-4065-86FD-C0FD95C7E89C}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>

</xml_diff>